<commit_message>
images for sentence completion task
starting to upload images for sentence completion task.
</commit_message>
<xml_diff>
--- a/stim/sentence_completion_task/sentence-completion_rhotic.xlsx
+++ b/stim/sentence_completion_task/sentence-completion_rhotic.xlsx
@@ -1,31 +1,42 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rober\Desktop\pt_in_newark\stim\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rober\Desktop\pt_in_newark\stim\sentence_completion_task\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF610EF8-7BB7-4180-8B61-FCA29E0E770B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3AE9067B-483C-4EC0-A22B-FB4520A73E51}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="296" uniqueCount="170">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="302" uniqueCount="176">
   <si>
     <t>lexical_item</t>
   </si>
@@ -549,12 +560,33 @@
   <si>
     <t>With gills, fish breathe.</t>
   </si>
+  <si>
+    <t>I listen to the radio to hear the latest news.</t>
+  </si>
+  <si>
+    <t>The queen is the king’s wife.</t>
+  </si>
+  <si>
+    <t>The beer bottle is full.</t>
+  </si>
+  <si>
+    <t>I want to eat a chocolate bar.</t>
+  </si>
+  <si>
+    <t>The car is red.</t>
+  </si>
+  <si>
+    <t>sentence_code</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <numFmts count="1">
+    <numFmt numFmtId="168" formatCode="00"/>
+  </numFmts>
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -566,6 +598,12 @@
       <i/>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -591,9 +629,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="168" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -874,1352 +913,1545 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H58"/>
+  <dimension ref="A1:I58"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="7" max="7" width="67.28515625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="57.42578125" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>175</v>
+      </c>
+      <c r="B1" t="s">
         <v>20</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>0</v>
       </c>
-      <c r="C1" t="s">
-        <v>1</v>
-      </c>
       <c r="D1" t="s">
+        <v>1</v>
+      </c>
+      <c r="E1" t="s">
         <v>2</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>3</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>17</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>18</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2" s="2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
         <v>21</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>5</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>6</v>
       </c>
-      <c r="D2">
-        <v>1</v>
-      </c>
       <c r="E2">
+        <v>1</v>
+      </c>
+      <c r="F2">
         <v>20020</v>
       </c>
-      <c r="F2" t="s">
+      <c r="G2" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
+      <c r="H2" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A3" s="2">
+        <v>2</v>
+      </c>
+      <c r="B3" t="s">
         <v>21</v>
       </c>
-      <c r="B3" t="s">
+      <c r="C3" t="s">
         <v>8</v>
       </c>
-      <c r="C3" t="s">
+      <c r="D3" t="s">
         <v>6</v>
       </c>
-      <c r="D3">
+      <c r="E3">
         <v>0</v>
       </c>
-      <c r="E3">
+      <c r="F3">
         <v>9207</v>
       </c>
-      <c r="F3" t="s">
+      <c r="G3" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+      <c r="H3" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A4" s="2">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
         <v>21</v>
       </c>
-      <c r="B4" t="s">
+      <c r="C4" t="s">
         <v>9</v>
       </c>
-      <c r="C4" t="s">
+      <c r="D4" t="s">
         <v>7</v>
       </c>
-      <c r="D4">
-        <v>1</v>
-      </c>
       <c r="E4">
+        <v>1</v>
+      </c>
+      <c r="F4">
         <v>8276</v>
       </c>
-      <c r="F4" t="s">
+      <c r="G4" t="s">
         <v>14</v>
       </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
+      <c r="H4" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A5" s="2">
+        <v>4</v>
+      </c>
+      <c r="B5" t="s">
         <v>21</v>
       </c>
-      <c r="B5" t="s">
+      <c r="C5" t="s">
         <v>10</v>
       </c>
-      <c r="C5" t="s">
+      <c r="D5" t="s">
         <v>7</v>
       </c>
-      <c r="D5">
+      <c r="E5">
         <v>0</v>
       </c>
-      <c r="E5">
+      <c r="F5">
         <v>10713</v>
       </c>
-      <c r="F5" t="s">
+      <c r="G5" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
+      <c r="H5" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A6" s="2">
+        <v>5</v>
+      </c>
+      <c r="B6" t="s">
         <v>21</v>
       </c>
-      <c r="B6" t="s">
+      <c r="C6" t="s">
         <v>11</v>
       </c>
-      <c r="C6" t="s">
+      <c r="D6" t="s">
         <v>7</v>
       </c>
-      <c r="D6">
+      <c r="E6">
         <v>0</v>
       </c>
-      <c r="E6">
+      <c r="F6">
         <v>62766</v>
       </c>
-      <c r="F6" t="s">
+      <c r="G6" t="s">
         <v>16</v>
       </c>
       <c r="H6" t="s">
+        <v>174</v>
+      </c>
+      <c r="I6" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A7" s="2">
+        <v>6</v>
+      </c>
+      <c r="B7" t="s">
         <v>22</v>
       </c>
-      <c r="B7" t="s">
+      <c r="C7" t="s">
         <v>23</v>
       </c>
-      <c r="C7" t="s">
+      <c r="D7" t="s">
         <v>24</v>
       </c>
-      <c r="D7">
-        <v>1</v>
-      </c>
-      <c r="E7" s="1">
+      <c r="E7">
+        <v>1</v>
+      </c>
+      <c r="F7" s="1">
         <v>3885</v>
       </c>
-      <c r="F7" t="s">
+      <c r="G7" t="s">
         <v>25</v>
       </c>
-      <c r="G7" t="s">
+      <c r="H7" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A8" s="2">
+        <v>7</v>
+      </c>
+      <c r="B8" t="s">
         <v>22</v>
       </c>
-      <c r="B8" t="s">
+      <c r="C8" t="s">
         <v>27</v>
       </c>
-      <c r="C8" t="s">
+      <c r="D8" t="s">
         <v>24</v>
       </c>
-      <c r="D8">
+      <c r="E8">
         <v>0</v>
       </c>
-      <c r="E8" s="1">
+      <c r="F8" s="1">
         <v>22483</v>
       </c>
-      <c r="F8" t="s">
+      <c r="G8" t="s">
         <v>28</v>
       </c>
-      <c r="G8" t="s">
+      <c r="H8" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A9" s="2">
+        <v>8</v>
+      </c>
+      <c r="B9" t="s">
         <v>22</v>
       </c>
-      <c r="B9" t="s">
+      <c r="C9" t="s">
         <v>30</v>
       </c>
-      <c r="C9" t="s">
+      <c r="D9" t="s">
         <v>24</v>
       </c>
-      <c r="D9">
+      <c r="E9">
         <v>0</v>
       </c>
-      <c r="E9" s="1">
+      <c r="F9" s="1">
         <v>9266</v>
       </c>
-      <c r="F9" t="s">
+      <c r="G9" t="s">
         <v>31</v>
       </c>
-      <c r="G9" t="s">
+      <c r="H9" t="s">
         <v>32</v>
       </c>
-      <c r="H9" t="s">
+      <c r="I9" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A10" s="2">
+        <v>9</v>
+      </c>
+      <c r="B10" t="s">
         <v>22</v>
       </c>
-      <c r="B10" t="s">
+      <c r="C10" t="s">
         <v>34</v>
       </c>
-      <c r="C10" t="s">
+      <c r="D10" t="s">
         <v>35</v>
       </c>
-      <c r="D10">
-        <v>1</v>
-      </c>
-      <c r="E10" s="1">
+      <c r="E10">
+        <v>1</v>
+      </c>
+      <c r="F10" s="1">
         <v>12754</v>
       </c>
-      <c r="F10" t="s">
+      <c r="G10" t="s">
         <v>36</v>
       </c>
-      <c r="G10" t="s">
+      <c r="H10" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A11" s="2">
+        <v>10</v>
+      </c>
+      <c r="B11" t="s">
         <v>22</v>
       </c>
-      <c r="B11" t="s">
+      <c r="C11" t="s">
         <v>38</v>
       </c>
-      <c r="C11" t="s">
+      <c r="D11" t="s">
         <v>35</v>
       </c>
-      <c r="D11">
+      <c r="E11">
         <v>0</v>
       </c>
-      <c r="E11" s="1">
+      <c r="F11" s="1">
         <v>129023</v>
       </c>
-      <c r="F11" t="s">
+      <c r="G11" t="s">
         <v>39</v>
       </c>
-      <c r="G11" t="s">
+      <c r="H11" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A12" s="2">
+        <v>11</v>
+      </c>
+      <c r="B12" t="s">
         <v>41</v>
       </c>
-      <c r="B12" t="s">
+      <c r="C12" t="s">
         <v>42</v>
       </c>
-      <c r="C12" t="s">
+      <c r="D12" t="s">
         <v>43</v>
       </c>
-      <c r="D12">
-        <v>1</v>
-      </c>
       <c r="E12">
+        <v>1</v>
+      </c>
+      <c r="F12">
         <v>23774</v>
       </c>
-      <c r="F12" t="s">
+      <c r="G12" t="s">
         <v>44</v>
       </c>
-      <c r="G12" t="s">
+      <c r="H12" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A13" s="2">
+        <v>12</v>
+      </c>
+      <c r="B13" t="s">
         <v>41</v>
       </c>
-      <c r="B13" t="s">
+      <c r="C13" t="s">
         <v>46</v>
       </c>
-      <c r="C13" t="s">
+      <c r="D13" t="s">
         <v>43</v>
       </c>
-      <c r="D13">
+      <c r="E13">
         <v>0</v>
       </c>
-      <c r="E13">
+      <c r="F13">
         <v>15274</v>
       </c>
-      <c r="F13" t="s">
+      <c r="G13" t="s">
         <v>47</v>
       </c>
-      <c r="G13" t="s">
+      <c r="H13" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A14" s="2">
+        <v>13</v>
+      </c>
+      <c r="B14" t="s">
         <v>41</v>
       </c>
-      <c r="B14" t="s">
+      <c r="C14" t="s">
         <v>49</v>
       </c>
-      <c r="C14" t="s">
+      <c r="D14" t="s">
         <v>43</v>
       </c>
-      <c r="D14">
-        <v>1</v>
-      </c>
       <c r="E14">
+        <v>1</v>
+      </c>
+      <c r="F14">
         <v>6195</v>
       </c>
-      <c r="F14" t="s">
+      <c r="G14" t="s">
         <v>50</v>
       </c>
-      <c r="G14" t="s">
+      <c r="H14" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A15" s="2">
+        <v>14</v>
+      </c>
+      <c r="B15" t="s">
         <v>41</v>
       </c>
-      <c r="B15" t="s">
+      <c r="C15" t="s">
         <v>52</v>
       </c>
-      <c r="C15" t="s">
+      <c r="D15" t="s">
         <v>43</v>
       </c>
-      <c r="D15">
+      <c r="E15">
         <v>0</v>
       </c>
-      <c r="E15">
+      <c r="F15">
         <v>8665</v>
       </c>
-      <c r="F15" t="s">
+      <c r="G15" t="s">
         <v>53</v>
       </c>
-      <c r="G15" t="s">
+      <c r="H15" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A16" s="2">
+        <v>15</v>
+      </c>
+      <c r="B16" t="s">
         <v>73</v>
       </c>
-      <c r="B16" t="s">
+      <c r="C16" t="s">
         <v>55</v>
       </c>
-      <c r="C16" t="s">
+      <c r="D16" t="s">
         <v>56</v>
       </c>
-      <c r="D16">
-        <v>1</v>
-      </c>
       <c r="E16">
+        <v>1</v>
+      </c>
+      <c r="F16">
         <v>21625</v>
       </c>
-      <c r="F16" t="s">
+      <c r="G16" t="s">
         <v>57</v>
       </c>
-      <c r="G16" t="s">
+      <c r="H16" t="s">
         <v>58</v>
       </c>
-      <c r="H16" t="s">
+      <c r="I16" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A17" s="2">
+        <v>16</v>
+      </c>
+      <c r="B17" t="s">
         <v>73</v>
       </c>
-      <c r="B17" t="s">
+      <c r="C17" t="s">
         <v>55</v>
       </c>
-      <c r="C17" t="s">
+      <c r="D17" t="s">
         <v>60</v>
       </c>
-      <c r="D17">
-        <v>1</v>
-      </c>
       <c r="E17">
+        <v>1</v>
+      </c>
+      <c r="F17">
         <v>21625</v>
       </c>
-      <c r="F17" t="s">
+      <c r="G17" t="s">
         <v>61</v>
       </c>
-      <c r="G17" t="s">
+      <c r="H17" t="s">
         <v>62</v>
       </c>
-      <c r="H17" t="s">
+      <c r="I17" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A18" s="2">
+        <v>17</v>
+      </c>
+      <c r="B18" t="s">
         <v>73</v>
       </c>
-      <c r="B18" t="s">
+      <c r="C18" t="s">
         <v>55</v>
       </c>
-      <c r="C18" t="s">
+      <c r="D18" t="s">
         <v>63</v>
       </c>
-      <c r="D18">
-        <v>1</v>
-      </c>
       <c r="E18">
+        <v>1</v>
+      </c>
+      <c r="F18">
         <v>21625</v>
       </c>
-      <c r="F18" t="s">
+      <c r="G18" t="s">
         <v>64</v>
       </c>
-      <c r="G18" t="s">
+      <c r="H18" t="s">
         <v>65</v>
       </c>
-      <c r="H18" t="s">
+      <c r="I18" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
+    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A19" s="2">
+        <v>18</v>
+      </c>
+      <c r="B19" t="s">
         <v>73</v>
       </c>
-      <c r="B19" t="s">
+      <c r="C19" t="s">
         <v>66</v>
       </c>
-      <c r="C19" t="s">
+      <c r="D19" t="s">
         <v>56</v>
       </c>
-      <c r="D19">
-        <v>1</v>
-      </c>
       <c r="E19">
+        <v>1</v>
+      </c>
+      <c r="F19">
         <v>10131</v>
       </c>
-      <c r="F19" t="s">
+      <c r="G19" t="s">
         <v>67</v>
       </c>
-      <c r="G19" t="s">
+      <c r="H19" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A20" s="2">
+        <v>19</v>
+      </c>
+      <c r="B20" t="s">
         <v>73</v>
       </c>
-      <c r="B20" t="s">
+      <c r="C20" t="s">
         <v>66</v>
       </c>
-      <c r="C20" t="s">
+      <c r="D20" t="s">
         <v>60</v>
       </c>
-      <c r="D20">
-        <v>1</v>
-      </c>
       <c r="E20">
+        <v>1</v>
+      </c>
+      <c r="F20">
         <v>10131</v>
       </c>
-      <c r="F20" t="s">
+      <c r="G20" t="s">
         <v>69</v>
       </c>
-      <c r="G20" t="s">
+      <c r="H20" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
+    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A21" s="2">
+        <v>20</v>
+      </c>
+      <c r="B21" t="s">
         <v>73</v>
       </c>
-      <c r="B21" t="s">
+      <c r="C21" t="s">
         <v>66</v>
       </c>
-      <c r="C21" t="s">
+      <c r="D21" t="s">
         <v>63</v>
       </c>
-      <c r="D21">
-        <v>1</v>
-      </c>
       <c r="E21">
+        <v>1</v>
+      </c>
+      <c r="F21">
         <v>10131</v>
       </c>
-      <c r="F21" t="s">
+      <c r="G21" t="s">
         <v>71</v>
       </c>
-      <c r="G21" t="s">
+      <c r="H21" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
+    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A22" s="2">
+        <v>21</v>
+      </c>
+      <c r="B22" t="s">
         <v>74</v>
       </c>
-      <c r="B22" t="s">
+      <c r="C22" t="s">
         <v>75</v>
       </c>
-      <c r="C22" t="s">
+      <c r="D22" t="s">
         <v>56</v>
       </c>
-      <c r="D22">
-        <v>1</v>
-      </c>
       <c r="E22">
+        <v>1</v>
+      </c>
+      <c r="F22">
         <v>70112</v>
       </c>
-      <c r="F22" t="s">
+      <c r="G22" t="s">
         <v>76</v>
       </c>
-      <c r="G22" t="s">
+      <c r="H22" t="s">
         <v>77</v>
       </c>
-      <c r="H22" t="s">
+      <c r="I22" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
+    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A23" s="2">
+        <v>22</v>
+      </c>
+      <c r="B23" t="s">
         <v>74</v>
       </c>
-      <c r="B23" t="s">
+      <c r="C23" t="s">
         <v>75</v>
       </c>
-      <c r="C23" t="s">
+      <c r="D23" t="s">
         <v>60</v>
       </c>
-      <c r="D23">
-        <v>1</v>
-      </c>
       <c r="E23">
+        <v>1</v>
+      </c>
+      <c r="F23">
         <v>70112</v>
       </c>
-      <c r="F23" t="s">
+      <c r="G23" t="s">
         <v>79</v>
       </c>
-      <c r="G23" t="s">
+      <c r="H23" t="s">
         <v>80</v>
       </c>
-      <c r="H23" t="s">
+      <c r="I23" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
+    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A24" s="2">
+        <v>23</v>
+      </c>
+      <c r="B24" t="s">
         <v>74</v>
       </c>
-      <c r="B24" t="s">
+      <c r="C24" t="s">
         <v>75</v>
       </c>
-      <c r="C24" t="s">
+      <c r="D24" t="s">
         <v>63</v>
       </c>
-      <c r="D24">
-        <v>1</v>
-      </c>
       <c r="E24">
+        <v>1</v>
+      </c>
+      <c r="F24">
         <v>70112</v>
       </c>
-      <c r="F24" t="s">
+      <c r="G24" t="s">
         <v>81</v>
       </c>
-      <c r="G24" t="s">
+      <c r="H24" t="s">
         <v>82</v>
       </c>
-      <c r="H24" t="s">
+      <c r="I24" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A25" t="s">
+    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A25" s="2">
+        <v>24</v>
+      </c>
+      <c r="B25" t="s">
         <v>74</v>
       </c>
-      <c r="B25" t="s">
+      <c r="C25" t="s">
         <v>83</v>
       </c>
-      <c r="C25" t="s">
+      <c r="D25" t="s">
         <v>56</v>
       </c>
-      <c r="D25">
-        <v>1</v>
-      </c>
       <c r="E25">
+        <v>1</v>
+      </c>
+      <c r="F25">
         <v>20532</v>
       </c>
-      <c r="F25" t="s">
+      <c r="G25" t="s">
         <v>84</v>
       </c>
-      <c r="G25" t="s">
+      <c r="H25" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A26" t="s">
+    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A26" s="2">
+        <v>25</v>
+      </c>
+      <c r="B26" t="s">
         <v>74</v>
       </c>
-      <c r="B26" t="s">
+      <c r="C26" t="s">
         <v>83</v>
       </c>
-      <c r="C26" t="s">
+      <c r="D26" t="s">
         <v>60</v>
       </c>
-      <c r="D26">
-        <v>1</v>
-      </c>
       <c r="E26">
+        <v>1</v>
+      </c>
+      <c r="F26">
         <v>20532</v>
       </c>
-      <c r="F26" t="s">
+      <c r="G26" t="s">
         <v>86</v>
       </c>
-      <c r="G26" t="s">
+      <c r="H26" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A27" t="s">
+    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A27" s="2">
+        <v>26</v>
+      </c>
+      <c r="B27" t="s">
         <v>74</v>
       </c>
-      <c r="B27" t="s">
+      <c r="C27" t="s">
         <v>83</v>
       </c>
-      <c r="C27" t="s">
+      <c r="D27" t="s">
         <v>63</v>
       </c>
-      <c r="D27">
-        <v>1</v>
-      </c>
       <c r="E27">
+        <v>1</v>
+      </c>
+      <c r="F27">
         <v>20532</v>
       </c>
-      <c r="F27" t="s">
+      <c r="G27" t="s">
         <v>88</v>
       </c>
-      <c r="G27" t="s">
+      <c r="H27" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A28" t="s">
+    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A28" s="2">
+        <v>27</v>
+      </c>
+      <c r="B28" t="s">
         <v>74</v>
       </c>
-      <c r="B28" t="s">
+      <c r="C28" t="s">
         <v>90</v>
       </c>
-      <c r="C28" t="s">
+      <c r="D28" t="s">
         <v>56</v>
       </c>
-      <c r="D28">
+      <c r="E28">
         <v>0</v>
       </c>
-      <c r="E28">
+      <c r="F28">
         <v>9801</v>
       </c>
-      <c r="F28" t="s">
+      <c r="G28" t="s">
         <v>91</v>
       </c>
-      <c r="G28" t="s">
+      <c r="H28" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A29" t="s">
+    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A29" s="2">
+        <v>28</v>
+      </c>
+      <c r="B29" t="s">
         <v>74</v>
       </c>
-      <c r="B29" t="s">
+      <c r="C29" t="s">
         <v>90</v>
       </c>
-      <c r="C29" t="s">
+      <c r="D29" t="s">
         <v>60</v>
       </c>
-      <c r="D29">
+      <c r="E29">
         <v>0</v>
       </c>
-      <c r="E29">
+      <c r="F29">
         <v>9801</v>
       </c>
-      <c r="F29" t="s">
+      <c r="G29" t="s">
         <v>93</v>
       </c>
-      <c r="G29" t="s">
+      <c r="H29" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A30" t="s">
+    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A30" s="2">
+        <v>29</v>
+      </c>
+      <c r="B30" t="s">
         <v>74</v>
       </c>
-      <c r="B30" t="s">
+      <c r="C30" t="s">
         <v>90</v>
       </c>
-      <c r="C30" t="s">
+      <c r="D30" t="s">
         <v>63</v>
       </c>
-      <c r="D30">
+      <c r="E30">
         <v>0</v>
       </c>
-      <c r="E30">
+      <c r="F30">
         <v>9801</v>
       </c>
-      <c r="F30" t="s">
+      <c r="G30" t="s">
         <v>95</v>
       </c>
-      <c r="G30" t="s">
+      <c r="H30" t="s">
         <v>96</v>
       </c>
     </row>
-    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A31" t="s">
+    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A31" s="2">
+        <v>30</v>
+      </c>
+      <c r="B31" t="s">
         <v>97</v>
       </c>
-      <c r="B31" t="s">
+      <c r="C31" t="s">
         <v>98</v>
       </c>
-      <c r="C31" t="s">
+      <c r="D31" t="s">
         <v>56</v>
       </c>
-      <c r="D31">
-        <v>1</v>
-      </c>
       <c r="E31">
+        <v>1</v>
+      </c>
+      <c r="F31">
         <v>119542</v>
       </c>
-      <c r="F31" t="s">
+      <c r="G31" t="s">
         <v>99</v>
       </c>
-      <c r="G31" t="s">
+      <c r="H31" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A32" t="s">
+    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A32" s="2">
+        <v>31</v>
+      </c>
+      <c r="B32" t="s">
         <v>97</v>
       </c>
-      <c r="B32" t="s">
+      <c r="C32" t="s">
         <v>98</v>
       </c>
-      <c r="C32" t="s">
+      <c r="D32" t="s">
         <v>60</v>
       </c>
-      <c r="D32">
-        <v>1</v>
-      </c>
       <c r="E32">
+        <v>1</v>
+      </c>
+      <c r="F32">
         <v>119542</v>
       </c>
-      <c r="F32" t="s">
+      <c r="G32" t="s">
         <v>101</v>
       </c>
-      <c r="G32" t="s">
+      <c r="H32" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A33" t="s">
+    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A33" s="2">
+        <v>32</v>
+      </c>
+      <c r="B33" t="s">
         <v>97</v>
       </c>
-      <c r="B33" t="s">
+      <c r="C33" t="s">
         <v>103</v>
       </c>
-      <c r="C33" t="s">
+      <c r="D33" t="s">
         <v>56</v>
       </c>
-      <c r="D33">
-        <v>1</v>
-      </c>
       <c r="E33">
+        <v>1</v>
+      </c>
+      <c r="F33">
         <v>175984</v>
       </c>
-      <c r="F33" t="s">
+      <c r="G33" t="s">
         <v>104</v>
       </c>
-      <c r="G33" t="s">
+      <c r="H33" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A34" t="s">
+    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A34" s="2">
+        <v>33</v>
+      </c>
+      <c r="B34" t="s">
         <v>97</v>
       </c>
-      <c r="B34" t="s">
+      <c r="C34" t="s">
         <v>103</v>
       </c>
-      <c r="C34" t="s">
+      <c r="D34" t="s">
         <v>60</v>
       </c>
-      <c r="D34">
-        <v>1</v>
-      </c>
       <c r="E34">
+        <v>1</v>
+      </c>
+      <c r="F34">
         <v>175984</v>
       </c>
-      <c r="F34" t="s">
+      <c r="G34" t="s">
         <v>106</v>
       </c>
-      <c r="G34" t="s">
+      <c r="H34" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A35" t="s">
+    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A35" s="2">
+        <v>34</v>
+      </c>
+      <c r="B35" t="s">
         <v>129</v>
       </c>
-      <c r="B35" t="s">
+      <c r="C35" t="s">
         <v>108</v>
       </c>
-      <c r="C35" t="s">
+      <c r="D35" t="s">
         <v>56</v>
       </c>
-      <c r="D35">
-        <v>1</v>
-      </c>
       <c r="E35">
+        <v>1</v>
+      </c>
+      <c r="F35">
         <v>69635</v>
       </c>
-      <c r="F35" t="s">
+      <c r="G35" t="s">
         <v>109</v>
       </c>
-      <c r="G35" t="s">
+      <c r="H35" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A36" t="s">
+    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A36" s="2">
+        <v>35</v>
+      </c>
+      <c r="B36" t="s">
         <v>129</v>
       </c>
-      <c r="B36" t="s">
+      <c r="C36" t="s">
         <v>108</v>
       </c>
-      <c r="C36" t="s">
+      <c r="D36" t="s">
         <v>60</v>
       </c>
-      <c r="D36">
-        <v>1</v>
-      </c>
       <c r="E36">
+        <v>1</v>
+      </c>
+      <c r="F36">
         <v>69635</v>
       </c>
-      <c r="F36" t="s">
+      <c r="G36" t="s">
         <v>111</v>
       </c>
-      <c r="G36" t="s">
+      <c r="H36" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A37" t="s">
+    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A37" s="2">
+        <v>36</v>
+      </c>
+      <c r="B37" t="s">
         <v>129</v>
       </c>
-      <c r="B37" t="s">
+      <c r="C37" t="s">
         <v>108</v>
       </c>
-      <c r="C37" t="s">
+      <c r="D37" t="s">
         <v>63</v>
       </c>
-      <c r="D37">
-        <v>1</v>
-      </c>
       <c r="E37">
+        <v>1</v>
+      </c>
+      <c r="F37">
         <v>69635</v>
       </c>
-      <c r="F37" t="s">
+      <c r="G37" t="s">
         <v>113</v>
       </c>
-      <c r="G37" t="s">
+      <c r="H37" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A38" t="s">
+    <row r="38" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A38" s="2">
+        <v>37</v>
+      </c>
+      <c r="B38" t="s">
         <v>129</v>
       </c>
-      <c r="B38" t="s">
+      <c r="C38" t="s">
         <v>115</v>
       </c>
-      <c r="C38" t="s">
+      <c r="D38" t="s">
         <v>56</v>
       </c>
-      <c r="D38">
-        <v>1</v>
-      </c>
       <c r="E38">
+        <v>1</v>
+      </c>
+      <c r="F38">
         <v>514408</v>
       </c>
-      <c r="F38" t="s">
+      <c r="G38" t="s">
         <v>116</v>
       </c>
-      <c r="G38" t="s">
+      <c r="H38" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A39" t="s">
+    <row r="39" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A39" s="2">
+        <v>38</v>
+      </c>
+      <c r="B39" t="s">
         <v>129</v>
       </c>
-      <c r="B39" t="s">
+      <c r="C39" t="s">
         <v>115</v>
       </c>
-      <c r="C39" t="s">
+      <c r="D39" t="s">
         <v>60</v>
       </c>
-      <c r="D39">
-        <v>1</v>
-      </c>
       <c r="E39">
+        <v>1</v>
+      </c>
+      <c r="F39">
         <v>514408</v>
       </c>
-      <c r="F39" t="s">
+      <c r="G39" t="s">
         <v>118</v>
       </c>
-      <c r="G39" t="s">
+      <c r="H39" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A40" t="s">
+    <row r="40" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A40" s="2">
+        <v>39</v>
+      </c>
+      <c r="B40" t="s">
         <v>129</v>
       </c>
-      <c r="B40" t="s">
+      <c r="C40" t="s">
         <v>115</v>
       </c>
-      <c r="C40" t="s">
+      <c r="D40" t="s">
         <v>63</v>
       </c>
-      <c r="D40">
-        <v>1</v>
-      </c>
       <c r="E40">
+        <v>1</v>
+      </c>
+      <c r="F40">
         <v>514408</v>
       </c>
-      <c r="F40" t="s">
+      <c r="G40" t="s">
         <v>120</v>
       </c>
-      <c r="G40" t="s">
+      <c r="H40" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A41" t="s">
+    <row r="41" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A41" s="2">
+        <v>40</v>
+      </c>
+      <c r="B41" t="s">
         <v>129</v>
       </c>
-      <c r="B41" t="s">
+      <c r="C41" t="s">
         <v>122</v>
       </c>
-      <c r="C41" t="s">
+      <c r="D41" t="s">
         <v>56</v>
       </c>
-      <c r="D41">
-        <v>1</v>
-      </c>
       <c r="E41">
+        <v>1</v>
+      </c>
+      <c r="F41">
         <v>38938</v>
       </c>
-      <c r="F41" t="s">
+      <c r="G41" t="s">
         <v>123</v>
       </c>
-      <c r="G41" t="s">
+      <c r="H41" t="s">
         <v>124</v>
       </c>
     </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A42" t="s">
+    <row r="42" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A42" s="2">
+        <v>41</v>
+      </c>
+      <c r="B42" t="s">
         <v>129</v>
       </c>
-      <c r="B42" t="s">
+      <c r="C42" t="s">
         <v>122</v>
       </c>
-      <c r="C42" t="s">
+      <c r="D42" t="s">
         <v>60</v>
       </c>
-      <c r="D42">
-        <v>1</v>
-      </c>
       <c r="E42">
+        <v>1</v>
+      </c>
+      <c r="F42">
         <v>38938</v>
       </c>
-      <c r="F42" t="s">
+      <c r="G42" t="s">
         <v>125</v>
       </c>
-      <c r="G42" t="s">
+      <c r="H42" t="s">
         <v>126</v>
       </c>
     </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A43" t="s">
+    <row r="43" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A43" s="2">
+        <v>42</v>
+      </c>
+      <c r="B43" t="s">
         <v>129</v>
       </c>
-      <c r="B43" t="s">
+      <c r="C43" t="s">
         <v>122</v>
       </c>
-      <c r="C43" t="s">
+      <c r="D43" t="s">
         <v>63</v>
       </c>
-      <c r="D43">
-        <v>1</v>
-      </c>
       <c r="E43">
+        <v>1</v>
+      </c>
+      <c r="F43">
         <v>38938</v>
       </c>
-      <c r="F43" t="s">
+      <c r="G43" t="s">
         <v>127</v>
       </c>
-      <c r="G43" t="s">
+      <c r="H43" t="s">
         <v>128</v>
       </c>
     </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A44" t="s">
+    <row r="44" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A44" s="2">
+        <v>43</v>
+      </c>
+      <c r="B44" t="s">
         <v>130</v>
       </c>
-      <c r="B44" t="s">
+      <c r="C44" t="s">
         <v>131</v>
       </c>
-      <c r="C44" t="s">
+      <c r="D44" t="s">
         <v>56</v>
       </c>
-      <c r="D44">
-        <v>1</v>
-      </c>
       <c r="E44">
+        <v>1</v>
+      </c>
+      <c r="F44">
         <v>39119</v>
       </c>
-      <c r="F44" t="s">
+      <c r="G44" t="s">
         <v>132</v>
       </c>
-      <c r="G44" t="s">
+      <c r="H44" t="s">
         <v>133</v>
       </c>
     </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A45" t="s">
+    <row r="45" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A45" s="2">
+        <v>44</v>
+      </c>
+      <c r="B45" t="s">
         <v>130</v>
       </c>
-      <c r="B45" t="s">
+      <c r="C45" t="s">
         <v>131</v>
       </c>
-      <c r="C45" t="s">
+      <c r="D45" t="s">
         <v>60</v>
       </c>
-      <c r="D45">
-        <v>1</v>
-      </c>
       <c r="E45">
+        <v>1</v>
+      </c>
+      <c r="F45">
         <v>39119</v>
       </c>
-      <c r="F45" t="s">
+      <c r="G45" t="s">
         <v>134</v>
       </c>
-      <c r="G45" t="s">
+      <c r="H45" t="s">
         <v>135</v>
       </c>
     </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A46" t="s">
+    <row r="46" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A46" s="2">
+        <v>45</v>
+      </c>
+      <c r="B46" t="s">
         <v>130</v>
       </c>
-      <c r="B46" t="s">
+      <c r="C46" t="s">
         <v>131</v>
       </c>
-      <c r="C46" t="s">
+      <c r="D46" t="s">
         <v>63</v>
       </c>
-      <c r="D46">
-        <v>1</v>
-      </c>
       <c r="E46">
+        <v>1</v>
+      </c>
+      <c r="F46">
         <v>39119</v>
       </c>
-      <c r="F46" t="s">
+      <c r="G46" t="s">
         <v>136</v>
       </c>
-      <c r="G46" t="s">
+      <c r="H46" t="s">
         <v>137</v>
       </c>
     </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A47" t="s">
+    <row r="47" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A47" s="2">
+        <v>46</v>
+      </c>
+      <c r="B47" t="s">
         <v>130</v>
       </c>
-      <c r="B47" t="s">
+      <c r="C47" t="s">
         <v>138</v>
       </c>
-      <c r="C47" t="s">
+      <c r="D47" t="s">
         <v>56</v>
       </c>
-      <c r="D47">
-        <v>1</v>
-      </c>
       <c r="E47">
+        <v>1</v>
+      </c>
+      <c r="F47">
         <v>165380</v>
       </c>
-      <c r="F47" t="s">
+      <c r="G47" t="s">
         <v>139</v>
       </c>
-      <c r="G47" t="s">
+      <c r="H47" t="s">
         <v>140</v>
       </c>
     </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A48" t="s">
+    <row r="48" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A48" s="2">
+        <v>47</v>
+      </c>
+      <c r="B48" t="s">
         <v>130</v>
       </c>
-      <c r="B48" t="s">
+      <c r="C48" t="s">
         <v>138</v>
       </c>
-      <c r="C48" t="s">
+      <c r="D48" t="s">
         <v>60</v>
       </c>
-      <c r="D48">
-        <v>1</v>
-      </c>
       <c r="E48">
+        <v>1</v>
+      </c>
+      <c r="F48">
         <v>165380</v>
       </c>
-      <c r="F48" t="s">
+      <c r="G48" t="s">
         <v>141</v>
       </c>
-      <c r="G48" t="s">
+      <c r="H48" t="s">
         <v>142</v>
       </c>
     </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A49" t="s">
+    <row r="49" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A49" s="2">
+        <v>48</v>
+      </c>
+      <c r="B49" t="s">
         <v>130</v>
       </c>
-      <c r="B49" t="s">
+      <c r="C49" t="s">
         <v>138</v>
       </c>
-      <c r="C49" t="s">
+      <c r="D49" t="s">
         <v>63</v>
       </c>
-      <c r="D49">
-        <v>1</v>
-      </c>
       <c r="E49">
+        <v>1</v>
+      </c>
+      <c r="F49">
         <v>165380</v>
       </c>
-      <c r="F49" t="s">
+      <c r="G49" t="s">
         <v>143</v>
       </c>
-      <c r="G49" t="s">
+      <c r="H49" t="s">
         <v>144</v>
       </c>
     </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A50" t="s">
+    <row r="50" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A50" s="2">
+        <v>49</v>
+      </c>
+      <c r="B50" t="s">
         <v>130</v>
       </c>
-      <c r="B50" t="s">
+      <c r="C50" t="s">
         <v>145</v>
       </c>
-      <c r="C50" t="s">
+      <c r="D50" t="s">
         <v>56</v>
       </c>
-      <c r="D50">
-        <v>1</v>
-      </c>
       <c r="E50">
+        <v>1</v>
+      </c>
+      <c r="F50">
         <v>30091</v>
       </c>
-      <c r="F50" t="s">
+      <c r="G50" t="s">
         <v>146</v>
       </c>
-      <c r="G50" t="s">
+      <c r="H50" t="s">
         <v>147</v>
       </c>
     </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A51" t="s">
+    <row r="51" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A51" s="2">
+        <v>50</v>
+      </c>
+      <c r="B51" t="s">
         <v>130</v>
       </c>
-      <c r="B51" t="s">
+      <c r="C51" t="s">
         <v>145</v>
       </c>
-      <c r="C51" t="s">
+      <c r="D51" t="s">
         <v>60</v>
       </c>
-      <c r="D51">
-        <v>1</v>
-      </c>
       <c r="E51">
+        <v>1</v>
+      </c>
+      <c r="F51">
         <v>30091</v>
       </c>
-      <c r="F51" t="s">
+      <c r="G51" t="s">
         <v>148</v>
       </c>
-      <c r="G51" t="s">
+      <c r="H51" t="s">
         <v>149</v>
       </c>
     </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A52" t="s">
+    <row r="52" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A52" s="2">
+        <v>51</v>
+      </c>
+      <c r="B52" t="s">
         <v>130</v>
       </c>
-      <c r="B52" t="s">
+      <c r="C52" t="s">
         <v>145</v>
       </c>
-      <c r="C52" t="s">
+      <c r="D52" t="s">
         <v>63</v>
       </c>
-      <c r="D52">
-        <v>1</v>
-      </c>
       <c r="E52">
+        <v>1</v>
+      </c>
+      <c r="F52">
         <v>30091</v>
       </c>
-      <c r="F52" t="s">
+      <c r="G52" t="s">
         <v>150</v>
       </c>
-      <c r="G52" t="s">
+      <c r="H52" t="s">
         <v>151</v>
       </c>
     </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A53" t="s">
+    <row r="53" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A53" s="2">
+        <v>52</v>
+      </c>
+      <c r="B53" t="s">
         <v>152</v>
       </c>
-      <c r="B53" t="s">
+      <c r="C53" t="s">
         <v>153</v>
       </c>
-      <c r="C53" t="s">
+      <c r="D53" t="s">
         <v>56</v>
       </c>
-      <c r="D53">
-        <v>1</v>
-      </c>
       <c r="E53">
+        <v>1</v>
+      </c>
+      <c r="F53">
         <v>87041</v>
       </c>
-      <c r="F53" t="s">
+      <c r="G53" t="s">
         <v>154</v>
       </c>
-      <c r="G53" t="s">
+      <c r="H53" t="s">
         <v>155</v>
       </c>
     </row>
-    <row r="54" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A54" t="s">
+    <row r="54" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A54" s="2">
+        <v>53</v>
+      </c>
+      <c r="B54" t="s">
         <v>152</v>
       </c>
-      <c r="B54" t="s">
+      <c r="C54" t="s">
         <v>153</v>
       </c>
-      <c r="C54" t="s">
+      <c r="D54" t="s">
         <v>60</v>
       </c>
-      <c r="D54">
-        <v>1</v>
-      </c>
       <c r="E54">
+        <v>1</v>
+      </c>
+      <c r="F54">
         <v>87041</v>
       </c>
-      <c r="F54" t="s">
+      <c r="G54" t="s">
         <v>156</v>
       </c>
-      <c r="G54" t="s">
+      <c r="H54" t="s">
         <v>157</v>
       </c>
     </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A55" t="s">
+    <row r="55" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A55" s="2">
+        <v>54</v>
+      </c>
+      <c r="B55" t="s">
         <v>152</v>
       </c>
-      <c r="B55" t="s">
+      <c r="C55" t="s">
         <v>158</v>
       </c>
-      <c r="C55" t="s">
+      <c r="D55" t="s">
         <v>56</v>
       </c>
-      <c r="D55">
-        <v>1</v>
-      </c>
       <c r="E55">
+        <v>1</v>
+      </c>
+      <c r="F55">
         <v>1273087</v>
       </c>
-      <c r="F55" t="s">
+      <c r="G55" t="s">
         <v>159</v>
       </c>
-      <c r="G55" t="s">
+      <c r="H55" t="s">
         <v>160</v>
       </c>
     </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A56" t="s">
+    <row r="56" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A56" s="2">
+        <v>55</v>
+      </c>
+      <c r="B56" t="s">
         <v>152</v>
       </c>
-      <c r="B56" t="s">
+      <c r="C56" t="s">
         <v>158</v>
       </c>
-      <c r="C56" t="s">
+      <c r="D56" t="s">
         <v>60</v>
       </c>
-      <c r="D56">
-        <v>1</v>
-      </c>
       <c r="E56">
+        <v>1</v>
+      </c>
+      <c r="F56">
         <v>1273087</v>
       </c>
-      <c r="F56" t="s">
+      <c r="G56" t="s">
         <v>161</v>
       </c>
-      <c r="G56" t="s">
+      <c r="H56" t="s">
         <v>162</v>
       </c>
     </row>
-    <row r="57" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A57" t="s">
+    <row r="57" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A57" s="2">
+        <v>56</v>
+      </c>
+      <c r="B57" t="s">
         <v>152</v>
       </c>
-      <c r="B57" t="s">
+      <c r="C57" t="s">
         <v>163</v>
       </c>
-      <c r="C57" t="s">
+      <c r="D57" t="s">
         <v>164</v>
       </c>
-      <c r="D57">
+      <c r="E57">
         <v>0</v>
       </c>
-      <c r="E57">
+      <c r="F57">
         <v>208</v>
       </c>
-      <c r="F57" t="s">
+      <c r="G57" t="s">
         <v>165</v>
       </c>
-      <c r="G57" t="s">
+      <c r="H57" t="s">
         <v>166</v>
       </c>
     </row>
-    <row r="58" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A58" t="s">
+    <row r="58" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A58" s="2">
+        <v>57</v>
+      </c>
+      <c r="B58" t="s">
         <v>152</v>
       </c>
-      <c r="B58" t="s">
+      <c r="C58" t="s">
         <v>167</v>
       </c>
-      <c r="C58" t="s">
+      <c r="D58" t="s">
         <v>164</v>
       </c>
-      <c r="D58">
+      <c r="E58">
         <v>0</v>
       </c>
-      <c r="E58">
+      <c r="F58">
         <v>24</v>
       </c>
-      <c r="F58" t="s">
+      <c r="G58" t="s">
         <v>168</v>
       </c>
-      <c r="G58" t="s">
+      <c r="H58" t="s">
         <v>169</v>
       </c>
     </row>

</xml_diff>